<commit_message>
Allow for local run
</commit_message>
<xml_diff>
--- a/output/similarity_matrix.xlsx
+++ b/output/similarity_matrix.xlsx
@@ -402,10 +402,10 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>0.8496976480285202</v>
+        <v>0.8836860903614391</v>
       </c>
       <c r="D2">
-        <v>0.883893145164005</v>
+        <v>0.9087452659631436</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -413,13 +413,13 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>0.8496976480285202</v>
+        <v>0.8836860903614391</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>0.7878396465991445</v>
+        <v>0.7902928321795319</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -427,10 +427,10 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>0.883893145164005</v>
+        <v>0.9087452659631436</v>
       </c>
       <c r="C4">
-        <v>0.7878396465991445</v>
+        <v>0.7902928321795319</v>
       </c>
       <c r="D4">
         <v>1</v>

</xml_diff>